<commit_message>
092325 - updated skins scoring.  did not post
</commit_message>
<xml_diff>
--- a/public/results/2025/2025 Weekly Stats - Week 21.xlsx
+++ b/public/results/2025/2025 Weekly Stats - Week 21.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\CODE\golf-league-site\public\results\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BABBD59-1D2F-44AE-8C0D-BDB5A9C9D775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D92BF23D-BCF1-4652-B3DC-D435157A03E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="930" yWindow="45" windowWidth="10785" windowHeight="10755" firstSheet="16" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="75" yWindow="30" windowWidth="19680" windowHeight="10755" firstSheet="16" activeTab="22" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="39" r:id="rId1"/>
@@ -419,7 +419,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -590,9 +590,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -24810,7 +24807,7 @@
         <f>IF(G17&gt;0, VLOOKUP(G17-G$5-(INT($M17/9)+(MOD($M17,9)&gt;=G$6)), 'Point System'!$A$4:$B$15, 2),"")</f>
         <v>1</v>
       </c>
-      <c r="H18" s="62">
+      <c r="H18" s="16">
         <f>IF(H17&gt;0, VLOOKUP(H17-H$5-(INT($M17/9)+(MOD($M17,9)&gt;=H$6)), 'Point System'!$A$4:$B$15, 2),"")</f>
         <v>3</v>
       </c>
@@ -24868,7 +24865,7 @@
       <c r="G19" s="12">
         <v>5</v>
       </c>
-      <c r="H19" s="12">
+      <c r="H19" s="46">
         <v>3</v>
       </c>
       <c r="I19" s="12">
@@ -25614,7 +25611,7 @@
         <v>3</v>
       </c>
       <c r="L32" s="17">
-        <f t="shared" ref="L31:L32" si="1">IF(SUM(C32:K32)&gt;0, SUM(C32:K32),"")</f>
+        <f t="shared" ref="L32" si="1">IF(SUM(C32:K32)&gt;0, SUM(C32:K32),"")</f>
         <v>23</v>
       </c>
       <c r="M32" s="16"/>

</xml_diff>